<commit_message>
Consulta por número da NF + série
- Bipagens passa a gravar NumeroNF (9 dígitos com zeros) e Serie (3 dígitos),
  extraídos da chave de acesso
- Nova tela Consultar NF: busca por número (com/sem zeros), série opcional
  ou chave bipada; mostra data, doca, itinerário, status e usuário
- Botão na tela inicial; modelo Excel, script e guia atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uf1Twg5uZphnaBMbSste1Z
</commit_message>
<xml_diff>
--- a/modelos/Expedicao_BancoDeDados.xlsx
+++ b/modelos/Expedicao_BancoDeDados.xlsx
@@ -155,9 +155,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Bipagens" displayName="Bipagens" ref="A1:J2" headerRowCount="1">
-  <autoFilter ref="A1:J2"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Bipagens" displayName="Bipagens" ref="A1:L2" headerRowCount="1">
+  <autoFilter ref="A1:L2"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="ChaveAcesso"/>
     <tableColumn id="2" name="Categoria"/>
     <tableColumn id="3" name="DataRef"/>
@@ -168,6 +168,8 @@
     <tableColumn id="8" name="Matricula"/>
     <tableColumn id="9" name="Usuario"/>
     <tableColumn id="10" name="Lote"/>
+    <tableColumn id="11" name="NumeroNF"/>
+    <tableColumn id="12" name="Serie"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -2174,7 +2176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2187,6 +2189,8 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2240,6 +2244,16 @@
           <t>Lote</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>NumeroNF</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2288,6 +2302,16 @@
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>exemplo</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>000000001</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
         </is>
       </c>
     </row>

</xml_diff>